<commit_message>
Funções de Banco de Dados
</commit_message>
<xml_diff>
--- a/Funções BD.xlsx
+++ b/Funções BD.xlsx
@@ -5,16 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edson.dpereira\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edson.dpereira\Documents\Excel Básico ao Avançado 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47B73D68-14DF-4198-BC7C-019F115A5E3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{253C98DA-8EE0-48A8-B04A-89D438EB1143}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Vendas - Funções BD" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="Banco">'Vendas - Funções BD'!$A$1:$H$102</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -681,8 +684,8 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="7" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="6" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="5" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -699,8 +702,8 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -939,28 +942,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="19" t="s">
+      <c r="E1" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="G1" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="19" t="s">
+      <c r="H1" s="13" t="s">
         <v>6</v>
       </c>
     </row>
@@ -986,7 +989,10 @@
       <c r="G2" s="3">
         <v>150</v>
       </c>
-      <c r="H2" s="3"/>
+      <c r="H2" s="3">
+        <f>F2*G2</f>
+        <v>1500</v>
+      </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -1010,7 +1016,10 @@
       <c r="G3" s="3">
         <v>800</v>
       </c>
-      <c r="H3" s="3"/>
+      <c r="H3" s="3">
+        <f t="shared" ref="H3:H66" si="0">F3*G3</f>
+        <v>3200</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -1034,7 +1043,10 @@
       <c r="G4" s="3">
         <v>150</v>
       </c>
-      <c r="H4" s="3"/>
+      <c r="H4" s="3">
+        <f t="shared" si="0"/>
+        <v>1200</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
@@ -1058,7 +1070,10 @@
       <c r="G5" s="3">
         <v>1200</v>
       </c>
-      <c r="H5" s="3"/>
+      <c r="H5" s="3">
+        <f t="shared" si="0"/>
+        <v>3600</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
@@ -1082,7 +1097,10 @@
       <c r="G6" s="3">
         <v>3500</v>
       </c>
-      <c r="H6" s="3"/>
+      <c r="H6" s="3">
+        <f t="shared" si="0"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
@@ -1106,7 +1124,10 @@
       <c r="G7" s="3">
         <v>1200</v>
       </c>
-      <c r="H7" s="3"/>
+      <c r="H7" s="3">
+        <f t="shared" si="0"/>
+        <v>2400</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
@@ -1130,7 +1151,10 @@
       <c r="G8" s="3">
         <v>1500</v>
       </c>
-      <c r="H8" s="3"/>
+      <c r="H8" s="3">
+        <f t="shared" si="0"/>
+        <v>3000</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
@@ -1154,7 +1178,10 @@
       <c r="G9" s="3">
         <v>80</v>
       </c>
-      <c r="H9" s="3"/>
+      <c r="H9" s="3">
+        <f t="shared" si="0"/>
+        <v>2000</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
@@ -1178,7 +1205,10 @@
       <c r="G10" s="3">
         <v>800</v>
       </c>
-      <c r="H10" s="3"/>
+      <c r="H10" s="3">
+        <f t="shared" si="0"/>
+        <v>4000</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
@@ -1202,7 +1232,10 @@
       <c r="G11" s="3">
         <v>3500</v>
       </c>
-      <c r="H11" s="3"/>
+      <c r="H11" s="3">
+        <f t="shared" si="0"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="12" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
@@ -1226,7 +1259,10 @@
       <c r="G12" s="3">
         <v>1500</v>
       </c>
-      <c r="H12" s="3"/>
+      <c r="H12" s="3">
+        <f t="shared" si="0"/>
+        <v>3000</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
@@ -1250,7 +1286,10 @@
       <c r="G13" s="3">
         <v>1200</v>
       </c>
-      <c r="H13" s="3"/>
+      <c r="H13" s="3">
+        <f t="shared" si="0"/>
+        <v>3600</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
@@ -1274,7 +1313,10 @@
       <c r="G14" s="3">
         <v>1200</v>
       </c>
-      <c r="H14" s="3"/>
+      <c r="H14" s="3">
+        <f t="shared" si="0"/>
+        <v>2400</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
@@ -1298,7 +1340,10 @@
       <c r="G15" s="3">
         <v>150</v>
       </c>
-      <c r="H15" s="3"/>
+      <c r="H15" s="3">
+        <f t="shared" si="0"/>
+        <v>1500</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
@@ -1322,7 +1367,10 @@
       <c r="G16" s="3">
         <v>3500</v>
       </c>
-      <c r="H16" s="3"/>
+      <c r="H16" s="3">
+        <f t="shared" si="0"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="17" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
@@ -1346,7 +1394,10 @@
       <c r="G17" s="3">
         <v>3500</v>
       </c>
-      <c r="H17" s="3"/>
+      <c r="H17" s="3">
+        <f t="shared" si="0"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="18" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
@@ -1370,7 +1421,10 @@
       <c r="G18" s="3">
         <v>1200</v>
       </c>
-      <c r="H18" s="3"/>
+      <c r="H18" s="3">
+        <f t="shared" si="0"/>
+        <v>2400</v>
+      </c>
     </row>
     <row r="19" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
@@ -1394,7 +1448,10 @@
       <c r="G19" s="3">
         <v>3500</v>
       </c>
-      <c r="H19" s="3"/>
+      <c r="H19" s="3">
+        <f t="shared" si="0"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="20" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
@@ -1418,7 +1475,10 @@
       <c r="G20" s="3">
         <v>1200</v>
       </c>
-      <c r="H20" s="3"/>
+      <c r="H20" s="3">
+        <f t="shared" si="0"/>
+        <v>1200</v>
+      </c>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
@@ -1442,7 +1502,10 @@
       <c r="G21" s="3">
         <v>3500</v>
       </c>
-      <c r="H21" s="3"/>
+      <c r="H21" s="3">
+        <f t="shared" si="0"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
@@ -1466,7 +1529,10 @@
       <c r="G22" s="3">
         <v>1200</v>
       </c>
-      <c r="H22" s="3"/>
+      <c r="H22" s="3">
+        <f t="shared" si="0"/>
+        <v>2400</v>
+      </c>
     </row>
     <row r="23" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
@@ -1490,7 +1556,10 @@
       <c r="G23" s="3">
         <v>1500</v>
       </c>
-      <c r="H23" s="3"/>
+      <c r="H23" s="3">
+        <f t="shared" si="0"/>
+        <v>1500</v>
+      </c>
     </row>
     <row r="24" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
@@ -1514,7 +1583,10 @@
       <c r="G24" s="3">
         <v>80</v>
       </c>
-      <c r="H24" s="3"/>
+      <c r="H24" s="3">
+        <f t="shared" si="0"/>
+        <v>800</v>
+      </c>
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
@@ -1538,7 +1610,10 @@
       <c r="G25" s="3">
         <v>800</v>
       </c>
-      <c r="H25" s="3"/>
+      <c r="H25" s="3">
+        <f t="shared" si="0"/>
+        <v>3200</v>
+      </c>
     </row>
     <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
@@ -1562,7 +1637,10 @@
       <c r="G26" s="3">
         <v>3500</v>
       </c>
-      <c r="H26" s="3"/>
+      <c r="H26" s="3">
+        <f t="shared" si="0"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="27" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
@@ -1586,7 +1664,10 @@
       <c r="G27" s="3">
         <v>1200</v>
       </c>
-      <c r="H27" s="3"/>
+      <c r="H27" s="3">
+        <f t="shared" si="0"/>
+        <v>6000</v>
+      </c>
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
@@ -1610,7 +1691,10 @@
       <c r="G28" s="3">
         <v>3500</v>
       </c>
-      <c r="H28" s="3"/>
+      <c r="H28" s="3">
+        <f t="shared" si="0"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
@@ -1634,7 +1718,10 @@
       <c r="G29" s="3">
         <v>1200</v>
       </c>
-      <c r="H29" s="3"/>
+      <c r="H29" s="3">
+        <f t="shared" si="0"/>
+        <v>2400</v>
+      </c>
     </row>
     <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
@@ -1658,7 +1745,10 @@
       <c r="G30" s="3">
         <v>800</v>
       </c>
-      <c r="H30" s="3"/>
+      <c r="H30" s="3">
+        <f t="shared" si="0"/>
+        <v>4800</v>
+      </c>
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
@@ -1682,7 +1772,10 @@
       <c r="G31" s="3">
         <v>80</v>
       </c>
-      <c r="H31" s="3"/>
+      <c r="H31" s="3">
+        <f t="shared" si="0"/>
+        <v>1600</v>
+      </c>
     </row>
     <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
@@ -1706,7 +1799,10 @@
       <c r="G32" s="3">
         <v>1500</v>
       </c>
-      <c r="H32" s="3"/>
+      <c r="H32" s="3">
+        <f t="shared" si="0"/>
+        <v>1500</v>
+      </c>
     </row>
     <row r="33" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
@@ -1730,7 +1826,10 @@
       <c r="G33" s="3">
         <v>3500</v>
       </c>
-      <c r="H33" s="3"/>
+      <c r="H33" s="3">
+        <f t="shared" si="0"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="34" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
@@ -1754,7 +1853,10 @@
       <c r="G34" s="3">
         <v>3500</v>
       </c>
-      <c r="H34" s="3"/>
+      <c r="H34" s="3">
+        <f t="shared" si="0"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
@@ -1778,7 +1880,10 @@
       <c r="G35" s="3">
         <v>1200</v>
       </c>
-      <c r="H35" s="3"/>
+      <c r="H35" s="3">
+        <f t="shared" si="0"/>
+        <v>3600</v>
+      </c>
     </row>
     <row r="36" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
@@ -1802,7 +1907,10 @@
       <c r="G36" s="3">
         <v>150</v>
       </c>
-      <c r="H36" s="3"/>
+      <c r="H36" s="3">
+        <f t="shared" si="0"/>
+        <v>2250</v>
+      </c>
     </row>
     <row r="37" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
@@ -1826,7 +1934,10 @@
       <c r="G37" s="3">
         <v>1200</v>
       </c>
-      <c r="H37" s="3"/>
+      <c r="H37" s="3">
+        <f t="shared" si="0"/>
+        <v>4800</v>
+      </c>
     </row>
     <row r="38" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
@@ -1850,7 +1961,10 @@
       <c r="G38" s="3">
         <v>3500</v>
       </c>
-      <c r="H38" s="3"/>
+      <c r="H38" s="3">
+        <f t="shared" si="0"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="39" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
@@ -1874,7 +1988,10 @@
       <c r="G39" s="3">
         <v>1500</v>
       </c>
-      <c r="H39" s="3"/>
+      <c r="H39" s="3">
+        <f t="shared" si="0"/>
+        <v>1500</v>
+      </c>
     </row>
     <row r="40" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
@@ -1898,7 +2015,10 @@
       <c r="G40" s="3">
         <v>1200</v>
       </c>
-      <c r="H40" s="3"/>
+      <c r="H40" s="3">
+        <f t="shared" si="0"/>
+        <v>6000</v>
+      </c>
     </row>
     <row r="41" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
@@ -1922,7 +2042,10 @@
       <c r="G41" s="3">
         <v>800</v>
       </c>
-      <c r="H41" s="3"/>
+      <c r="H41" s="3">
+        <f t="shared" si="0"/>
+        <v>1600</v>
+      </c>
     </row>
     <row r="42" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
@@ -1946,7 +2069,10 @@
       <c r="G42" s="3">
         <v>80</v>
       </c>
-      <c r="H42" s="3"/>
+      <c r="H42" s="3">
+        <f t="shared" si="0"/>
+        <v>1200</v>
+      </c>
     </row>
     <row r="43" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
@@ -1970,7 +2096,10 @@
       <c r="G43" s="3">
         <v>1500</v>
       </c>
-      <c r="H43" s="3"/>
+      <c r="H43" s="3">
+        <f t="shared" si="0"/>
+        <v>1500</v>
+      </c>
     </row>
     <row r="44" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
@@ -1994,7 +2123,10 @@
       <c r="G44" s="3">
         <v>80</v>
       </c>
-      <c r="H44" s="3"/>
+      <c r="H44" s="3">
+        <f t="shared" si="0"/>
+        <v>800</v>
+      </c>
     </row>
     <row r="45" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
@@ -2018,7 +2150,10 @@
       <c r="G45" s="3">
         <v>800</v>
       </c>
-      <c r="H45" s="3"/>
+      <c r="H45" s="3">
+        <f t="shared" si="0"/>
+        <v>2400</v>
+      </c>
     </row>
     <row r="46" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
@@ -2042,7 +2177,10 @@
       <c r="G46" s="3">
         <v>80</v>
       </c>
-      <c r="H46" s="3"/>
+      <c r="H46" s="3">
+        <f t="shared" si="0"/>
+        <v>1600</v>
+      </c>
     </row>
     <row r="47" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
@@ -2066,7 +2204,10 @@
       <c r="G47" s="3">
         <v>1500</v>
       </c>
-      <c r="H47" s="3"/>
+      <c r="H47" s="3">
+        <f t="shared" si="0"/>
+        <v>1500</v>
+      </c>
     </row>
     <row r="48" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
@@ -2090,7 +2231,10 @@
       <c r="G48" s="3">
         <v>3500</v>
       </c>
-      <c r="H48" s="3"/>
+      <c r="H48" s="3">
+        <f t="shared" si="0"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="49" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
@@ -2114,7 +2258,10 @@
       <c r="G49" s="3">
         <v>3500</v>
       </c>
-      <c r="H49" s="3"/>
+      <c r="H49" s="3">
+        <f t="shared" si="0"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="50" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
@@ -2138,7 +2285,10 @@
       <c r="G50" s="3">
         <v>1200</v>
       </c>
-      <c r="H50" s="3"/>
+      <c r="H50" s="3">
+        <f t="shared" si="0"/>
+        <v>2400</v>
+      </c>
     </row>
     <row r="51" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
@@ -2162,7 +2312,10 @@
       <c r="G51" s="3">
         <v>150</v>
       </c>
-      <c r="H51" s="3"/>
+      <c r="H51" s="3">
+        <f t="shared" si="0"/>
+        <v>1500</v>
+      </c>
     </row>
     <row r="52" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
@@ -2186,7 +2339,10 @@
       <c r="G52" s="3">
         <v>80</v>
       </c>
-      <c r="H52" s="3"/>
+      <c r="H52" s="3">
+        <f t="shared" si="0"/>
+        <v>1200</v>
+      </c>
     </row>
     <row r="53" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
@@ -2210,7 +2366,10 @@
       <c r="G53" s="3">
         <v>1500</v>
       </c>
-      <c r="H53" s="3"/>
+      <c r="H53" s="3">
+        <f t="shared" si="0"/>
+        <v>3000</v>
+      </c>
     </row>
     <row r="54" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
@@ -2234,7 +2393,10 @@
       <c r="G54" s="3">
         <v>80</v>
       </c>
-      <c r="H54" s="3"/>
+      <c r="H54" s="3">
+        <f t="shared" si="0"/>
+        <v>960</v>
+      </c>
     </row>
     <row r="55" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
@@ -2258,7 +2420,10 @@
       <c r="G55" s="3">
         <v>3500</v>
       </c>
-      <c r="H55" s="3"/>
+      <c r="H55" s="3">
+        <f t="shared" si="0"/>
+        <v>7000</v>
+      </c>
     </row>
     <row r="56" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
@@ -2282,7 +2447,10 @@
       <c r="G56" s="3">
         <v>1200</v>
       </c>
-      <c r="H56" s="3"/>
+      <c r="H56" s="3">
+        <f t="shared" si="0"/>
+        <v>4800</v>
+      </c>
     </row>
     <row r="57" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
@@ -2306,7 +2474,10 @@
       <c r="G57" s="3">
         <v>150</v>
       </c>
-      <c r="H57" s="3"/>
+      <c r="H57" s="3">
+        <f t="shared" si="0"/>
+        <v>1500</v>
+      </c>
     </row>
     <row r="58" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
@@ -2330,7 +2501,10 @@
       <c r="G58" s="3">
         <v>800</v>
       </c>
-      <c r="H58" s="3"/>
+      <c r="H58" s="3">
+        <f t="shared" si="0"/>
+        <v>2400</v>
+      </c>
     </row>
     <row r="59" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
@@ -2354,7 +2528,10 @@
       <c r="G59" s="3">
         <v>150</v>
       </c>
-      <c r="H59" s="3"/>
+      <c r="H59" s="3">
+        <f t="shared" si="0"/>
+        <v>1500</v>
+      </c>
     </row>
     <row r="60" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
@@ -2378,7 +2555,10 @@
       <c r="G60" s="3">
         <v>1500</v>
       </c>
-      <c r="H60" s="3"/>
+      <c r="H60" s="3">
+        <f t="shared" si="0"/>
+        <v>1500</v>
+      </c>
     </row>
     <row r="61" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
@@ -2402,7 +2582,10 @@
       <c r="G61" s="3">
         <v>80</v>
       </c>
-      <c r="H61" s="3"/>
+      <c r="H61" s="3">
+        <f t="shared" si="0"/>
+        <v>2400</v>
+      </c>
     </row>
     <row r="62" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
@@ -2426,7 +2609,10 @@
       <c r="G62" s="3">
         <v>800</v>
       </c>
-      <c r="H62" s="3"/>
+      <c r="H62" s="3">
+        <f t="shared" si="0"/>
+        <v>3200</v>
+      </c>
     </row>
     <row r="63" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
@@ -2450,7 +2636,10 @@
       <c r="G63" s="3">
         <v>150</v>
       </c>
-      <c r="H63" s="3"/>
+      <c r="H63" s="3">
+        <f t="shared" si="0"/>
+        <v>1800</v>
+      </c>
     </row>
     <row r="64" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
@@ -2474,7 +2663,10 @@
       <c r="G64" s="3">
         <v>3500</v>
       </c>
-      <c r="H64" s="3"/>
+      <c r="H64" s="3">
+        <f t="shared" si="0"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="65" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
@@ -2498,7 +2690,10 @@
       <c r="G65" s="3">
         <v>3500</v>
       </c>
-      <c r="H65" s="3"/>
+      <c r="H65" s="3">
+        <f t="shared" si="0"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="66" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
@@ -2522,7 +2717,10 @@
       <c r="G66" s="3">
         <v>1200</v>
       </c>
-      <c r="H66" s="3"/>
+      <c r="H66" s="3">
+        <f t="shared" si="0"/>
+        <v>2400</v>
+      </c>
     </row>
     <row r="67" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
@@ -2546,7 +2744,10 @@
       <c r="G67" s="3">
         <v>1200</v>
       </c>
-      <c r="H67" s="3"/>
+      <c r="H67" s="3">
+        <f t="shared" ref="H67:H102" si="1">F67*G67</f>
+        <v>3600</v>
+      </c>
     </row>
     <row r="68" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
@@ -2570,7 +2771,10 @@
       <c r="G68" s="3">
         <v>3500</v>
       </c>
-      <c r="H68" s="3"/>
+      <c r="H68" s="3">
+        <f t="shared" si="1"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="69" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
@@ -2594,7 +2798,10 @@
       <c r="G69" s="3">
         <v>1200</v>
       </c>
-      <c r="H69" s="3"/>
+      <c r="H69" s="3">
+        <f t="shared" si="1"/>
+        <v>4800</v>
+      </c>
     </row>
     <row r="70" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
@@ -2618,7 +2825,10 @@
       <c r="G70" s="3">
         <v>3500</v>
       </c>
-      <c r="H70" s="3"/>
+      <c r="H70" s="3">
+        <f t="shared" si="1"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="71" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
@@ -2642,7 +2852,10 @@
       <c r="G71" s="3">
         <v>1200</v>
       </c>
-      <c r="H71" s="3"/>
+      <c r="H71" s="3">
+        <f t="shared" si="1"/>
+        <v>3600</v>
+      </c>
     </row>
     <row r="72" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
@@ -2666,7 +2879,10 @@
       <c r="G72" s="3">
         <v>150</v>
       </c>
-      <c r="H72" s="3"/>
+      <c r="H72" s="3">
+        <f t="shared" si="1"/>
+        <v>2250</v>
+      </c>
     </row>
     <row r="73" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
@@ -2690,7 +2906,10 @@
       <c r="G73" s="3">
         <v>800</v>
       </c>
-      <c r="H73" s="3"/>
+      <c r="H73" s="3">
+        <f t="shared" si="1"/>
+        <v>1600</v>
+      </c>
     </row>
     <row r="74" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
@@ -2714,7 +2933,10 @@
       <c r="G74" s="3">
         <v>150</v>
       </c>
-      <c r="H74" s="3"/>
+      <c r="H74" s="3">
+        <f t="shared" si="1"/>
+        <v>750</v>
+      </c>
     </row>
     <row r="75" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
@@ -2738,7 +2960,10 @@
       <c r="G75" s="3">
         <v>1500</v>
       </c>
-      <c r="H75" s="3"/>
+      <c r="H75" s="3">
+        <f t="shared" si="1"/>
+        <v>3000</v>
+      </c>
     </row>
     <row r="76" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
@@ -2762,7 +2987,10 @@
       <c r="G76" s="3">
         <v>80</v>
       </c>
-      <c r="H76" s="3"/>
+      <c r="H76" s="3">
+        <f t="shared" si="1"/>
+        <v>1600</v>
+      </c>
     </row>
     <row r="77" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
@@ -2786,7 +3014,10 @@
       <c r="G77" s="3">
         <v>3500</v>
       </c>
-      <c r="H77" s="3"/>
+      <c r="H77" s="3">
+        <f t="shared" si="1"/>
+        <v>7000</v>
+      </c>
     </row>
     <row r="78" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
@@ -2810,7 +3041,10 @@
       <c r="G78" s="3">
         <v>1200</v>
       </c>
-      <c r="H78" s="3"/>
+      <c r="H78" s="3">
+        <f t="shared" si="1"/>
+        <v>3600</v>
+      </c>
     </row>
     <row r="79" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
@@ -2834,7 +3068,10 @@
       <c r="G79" s="3">
         <v>3500</v>
       </c>
-      <c r="H79" s="3"/>
+      <c r="H79" s="3">
+        <f t="shared" si="1"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="80" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
@@ -2858,7 +3095,10 @@
       <c r="G80" s="3">
         <v>1500</v>
       </c>
-      <c r="H80" s="3"/>
+      <c r="H80" s="3">
+        <f t="shared" si="1"/>
+        <v>1500</v>
+      </c>
     </row>
     <row r="81" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
@@ -2882,7 +3122,10 @@
       <c r="G81" s="3">
         <v>150</v>
       </c>
-      <c r="H81" s="3"/>
+      <c r="H81" s="3">
+        <f t="shared" si="1"/>
+        <v>750</v>
+      </c>
     </row>
     <row r="82" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
@@ -2906,7 +3149,10 @@
       <c r="G82" s="3">
         <v>800</v>
       </c>
-      <c r="H82" s="3"/>
+      <c r="H82" s="3">
+        <f t="shared" si="1"/>
+        <v>1600</v>
+      </c>
     </row>
     <row r="83" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
@@ -2930,7 +3176,10 @@
       <c r="G83" s="3">
         <v>80</v>
       </c>
-      <c r="H83" s="3"/>
+      <c r="H83" s="3">
+        <f t="shared" si="1"/>
+        <v>1200</v>
+      </c>
     </row>
     <row r="84" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
@@ -2954,7 +3203,10 @@
       <c r="G84" s="3">
         <v>1200</v>
       </c>
-      <c r="H84" s="3"/>
+      <c r="H84" s="3">
+        <f t="shared" si="1"/>
+        <v>4800</v>
+      </c>
     </row>
     <row r="85" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
@@ -2978,7 +3230,10 @@
       <c r="G85" s="3">
         <v>3500</v>
       </c>
-      <c r="H85" s="3"/>
+      <c r="H85" s="3">
+        <f t="shared" si="1"/>
+        <v>7000</v>
+      </c>
     </row>
     <row r="86" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
@@ -3002,7 +3257,10 @@
       <c r="G86" s="3">
         <v>1200</v>
       </c>
-      <c r="H86" s="3"/>
+      <c r="H86" s="3">
+        <f t="shared" si="1"/>
+        <v>2400</v>
+      </c>
     </row>
     <row r="87" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
@@ -3026,7 +3284,10 @@
       <c r="G87" s="3">
         <v>3500</v>
       </c>
-      <c r="H87" s="3"/>
+      <c r="H87" s="3">
+        <f t="shared" si="1"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="88" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
@@ -3050,7 +3311,10 @@
       <c r="G88" s="3">
         <v>80</v>
       </c>
-      <c r="H88" s="3"/>
+      <c r="H88" s="3">
+        <f t="shared" si="1"/>
+        <v>800</v>
+      </c>
     </row>
     <row r="89" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
@@ -3074,7 +3338,10 @@
       <c r="G89" s="3">
         <v>800</v>
       </c>
-      <c r="H89" s="3"/>
+      <c r="H89" s="3">
+        <f t="shared" si="1"/>
+        <v>2400</v>
+      </c>
     </row>
     <row r="90" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
@@ -3098,7 +3365,10 @@
       <c r="G90" s="3">
         <v>80</v>
       </c>
-      <c r="H90" s="3"/>
+      <c r="H90" s="3">
+        <f t="shared" si="1"/>
+        <v>1600</v>
+      </c>
     </row>
     <row r="91" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
@@ -3122,7 +3392,10 @@
       <c r="G91" s="3">
         <v>1500</v>
       </c>
-      <c r="H91" s="3"/>
+      <c r="H91" s="3">
+        <f t="shared" si="1"/>
+        <v>1500</v>
+      </c>
     </row>
     <row r="92" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
@@ -3146,7 +3419,10 @@
       <c r="G92" s="3">
         <v>150</v>
       </c>
-      <c r="H92" s="3"/>
+      <c r="H92" s="3">
+        <f t="shared" si="1"/>
+        <v>900</v>
+      </c>
     </row>
     <row r="93" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
@@ -3170,7 +3446,10 @@
       <c r="G93" s="3">
         <v>800</v>
       </c>
-      <c r="H93" s="3"/>
+      <c r="H93" s="3">
+        <f t="shared" si="1"/>
+        <v>3200</v>
+      </c>
     </row>
     <row r="94" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
@@ -3194,7 +3473,10 @@
       <c r="G94" s="3">
         <v>150</v>
       </c>
-      <c r="H94" s="3"/>
+      <c r="H94" s="3">
+        <f t="shared" si="1"/>
+        <v>1200</v>
+      </c>
     </row>
     <row r="95" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
@@ -3218,7 +3500,10 @@
       <c r="G95" s="3">
         <v>1500</v>
       </c>
-      <c r="H95" s="3"/>
+      <c r="H95" s="3">
+        <f t="shared" si="1"/>
+        <v>3000</v>
+      </c>
     </row>
     <row r="96" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
@@ -3242,7 +3527,10 @@
       <c r="G96" s="3">
         <v>150</v>
       </c>
-      <c r="H96" s="3"/>
+      <c r="H96" s="3">
+        <f t="shared" si="1"/>
+        <v>1500</v>
+      </c>
     </row>
     <row r="97" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
@@ -3266,7 +3554,10 @@
       <c r="G97" s="3">
         <v>800</v>
       </c>
-      <c r="H97" s="3"/>
+      <c r="H97" s="3">
+        <f t="shared" si="1"/>
+        <v>4000</v>
+      </c>
     </row>
     <row r="98" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
@@ -3290,7 +3581,10 @@
       <c r="G98" s="3">
         <v>80</v>
       </c>
-      <c r="H98" s="3"/>
+      <c r="H98" s="3">
+        <f t="shared" si="1"/>
+        <v>960</v>
+      </c>
     </row>
     <row r="99" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
@@ -3314,7 +3608,10 @@
       <c r="G99" s="3">
         <v>1200</v>
       </c>
-      <c r="H99" s="3"/>
+      <c r="H99" s="3">
+        <f t="shared" si="1"/>
+        <v>3600</v>
+      </c>
     </row>
     <row r="100" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
@@ -3338,7 +3635,10 @@
       <c r="G100" s="3">
         <v>3500</v>
       </c>
-      <c r="H100" s="3"/>
+      <c r="H100" s="3">
+        <f t="shared" si="1"/>
+        <v>3500</v>
+      </c>
     </row>
     <row r="101" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
@@ -3362,7 +3662,10 @@
       <c r="G101" s="3">
         <v>1200</v>
       </c>
-      <c r="H101" s="3"/>
+      <c r="H101" s="3">
+        <f t="shared" si="1"/>
+        <v>1200</v>
+      </c>
     </row>
     <row r="102" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="5" t="s">
@@ -3386,16 +3689,19 @@
       <c r="G102" s="3">
         <v>3500</v>
       </c>
-      <c r="H102" s="3"/>
-    </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H102" s="3">
+        <f t="shared" si="1"/>
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A105" s="18" t="s">
         <v>23</v>
       </c>
       <c r="B105" s="18"/>
       <c r="C105" s="18"/>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A106" s="7" t="s">
         <v>0</v>
       </c>
@@ -3407,11 +3713,11 @@
       </c>
     </row>
     <row r="107" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A107" s="5"/>
+      <c r="A107" s="1"/>
       <c r="B107" s="1"/>
       <c r="C107" s="1"/>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A109" s="17" t="s">
         <v>24</v>
       </c>
@@ -3419,7 +3725,7 @@
       <c r="C109" s="17"/>
       <c r="D109" s="17"/>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A110" s="7" t="s">
         <v>25</v>
       </c>
@@ -3433,87 +3739,129 @@
       <c r="A111" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B111" s="13" t="s">
+      <c r="B111" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="C111" s="13"/>
-      <c r="D111" s="3"/>
+      <c r="C111" s="19"/>
+      <c r="D111" s="3">
+        <f>DSUM(Banco,$H$1,$A$106:$C$107)</f>
+        <v>275920</v>
+      </c>
+      <c r="E111" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(D111)</f>
+        <v>=BDSOMA(Banco;$H$1;$A$106:$C$107)</v>
+      </c>
     </row>
     <row r="112" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B112" s="13" t="s">
+      <c r="B112" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="C112" s="13"/>
-      <c r="D112" s="3"/>
-    </row>
-    <row r="113" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C112" s="19"/>
+      <c r="D112" s="3">
+        <f>DAVERAGE(Banco,"Quantidade",$A$106:$C$107)</f>
+        <v>5.1980198019801982</v>
+      </c>
+      <c r="E112" t="str">
+        <f t="shared" ref="E112:E117" ca="1" si="2">_xlfn.FORMULATEXT(D112)</f>
+        <v>=BDMÉDIA(Banco;"Quantidade";$A$106:$C$107)</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B113" s="13" t="s">
+      <c r="B113" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="C113" s="13"/>
-      <c r="D113" s="3"/>
-    </row>
-    <row r="114" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C113" s="19"/>
+      <c r="D113" s="3">
+        <f>DMAX(Banco,"Preço Unitário",$A$106:$C$107)</f>
+        <v>3500</v>
+      </c>
+      <c r="E113" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>=BDMÁX(Banco;"Preço Unitário";$A$106:$C$107)</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B114" s="13" t="s">
+      <c r="B114" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="C114" s="13"/>
-      <c r="D114" s="3"/>
-    </row>
-    <row r="115" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C114" s="19"/>
+      <c r="D114" s="3">
+        <f>DMIN(Banco,"Preço Unitário",$A$106:$C$107)</f>
+        <v>80</v>
+      </c>
+      <c r="E114" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>=BDMÍN(Banco;"Preço Unitário";$A$106:$C$107)</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B115" s="13" t="s">
+      <c r="B115" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="C115" s="13"/>
-      <c r="D115" s="1"/>
-    </row>
-    <row r="116" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C115" s="19"/>
+      <c r="D115" s="3"/>
+    </row>
+    <row r="116" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B116" s="13" t="s">
+      <c r="B116" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="C116" s="13"/>
-      <c r="D116" s="8"/>
-    </row>
-    <row r="117" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C116" s="19"/>
+      <c r="D116" s="8">
+        <f>DCOUNT(Banco,$H$1,$A$106:$C$107)</f>
+        <v>101</v>
+      </c>
+      <c r="E116" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>=BDCONTAR(Banco;$H$1;$A$106:$C$107)</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B117" s="13" t="s">
+      <c r="B117" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="C117" s="13"/>
-      <c r="D117" s="8"/>
+      <c r="C117" s="19"/>
+      <c r="D117" s="8">
+        <f>DCOUNTA(Banco,$H$1,$A$106:$C$107)</f>
+        <v>101</v>
+      </c>
+      <c r="E117" t="str">
+        <f t="shared" ca="1" si="2"/>
+        <v>=BDCONTARA(Banco;$H$1;$A$106:$C$107)</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G102">
     <sortCondition ref="B2:B102"/>
   </sortState>
   <mergeCells count="10">
+    <mergeCell ref="B115:C115"/>
+    <mergeCell ref="B116:C116"/>
+    <mergeCell ref="B117:C117"/>
+    <mergeCell ref="B113:C113"/>
+    <mergeCell ref="B114:C114"/>
     <mergeCell ref="B110:D110"/>
     <mergeCell ref="A109:D109"/>
     <mergeCell ref="A105:C105"/>
     <mergeCell ref="B111:C111"/>
     <mergeCell ref="B112:C112"/>
-    <mergeCell ref="B115:C115"/>
-    <mergeCell ref="B116:C116"/>
-    <mergeCell ref="B117:C117"/>
-    <mergeCell ref="B113:C113"/>
-    <mergeCell ref="B114:C114"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>